<commit_message>
Plan xlsx: irrigation items now IN CI (PR open)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T49gnSNZq31rPRt1vHk4Rc
</commit_message>
<xml_diff>
--- a/nexidoc/plans/Nexi_Requests_9Oct2026_Status_and_Plan.xlsx
+++ b/nexidoc/plans/Nexi_Requests_9Oct2026_Status_and_Plan.xlsx
@@ -711,12 +711,12 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>BUILT on branch hotfix/irr-pool (worktree wf_aa1e5c2b-673-6): 5 commits + 5 files uncommitted (the first-pull race gate - finished, syntax OK, not yet committed). Suite on next.html 20/22; the 2 red are test-side (date mask / 11-s wait). Review r1: 8 must-fix, all addressed in round 2; final review not finished.</t>
+          <t>BUILT on branch hotfix/irr-pool (worktree wf_aa1e5c2b-673-6): 5 commits + 5 files uncommitted (the first-pull race gate - finished, syntax OK, not yet committed). Suite on next.html 20/22; the 2 red are test-side (date mask / 11-s wait). Review r1: 8 must-fix, all addressed in round 2; final review not finished. | 10:30: gate committed (c2d00ee); the 2 red cases now GREEN on both pages; branch merged to the working branch (4852cb3); PR opened; CI 25 jobs running.</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>BUILT - NOT YET LIVE</t>
+          <t>IN CI - PR OPEN (merge when green)</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -761,12 +761,12 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>IN the same branch: IRR_LEVEL_BANDS_BY_GH + EC/pH bands seeded exactly as you wrote; the old private _IRR_RANGES (EC 1.2-3.2 / pH 5.5-6.5) deleted. Test "🎨 Eyal's ranges" passes at every boundary (1.49 crit, 1.50 warn, 1.69 warn, 1.70 ok, 1.90 ok, 1.91 warn, 2.00 warn, 2.01 crit ...).</t>
+          <t>IN the same branch: IRR_LEVEL_BANDS_BY_GH + EC/pH bands seeded exactly as you wrote; the old private _IRR_RANGES (EC 1.2-3.2 / pH 5.5-6.5) deleted. Test "🎨 Eyal's ranges" passes at every boundary (1.49 crit, 1.50 warn, 1.69 warn, 1.70 ok, 1.90 ok, 1.91 warn, 2.00 warn, 2.01 crit ...). | 10:30: gate committed (c2d00ee); the 2 red cases now GREEN on both pages; branch merged to the working branch (4852cb3); PR opened; CI 25 jobs running.</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
         <is>
-          <t>BUILT - NOT YET LIVE</t>
+          <t>IN CI - PR OPEN (merge when green)</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -811,12 +811,12 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>IN the same branch: IRR_DAILY_TARGET_BY_GH exactly as you wrote; dim.target kept as the cleaning level; Smart Dosing uses the same engine (Pool 1 at 54 cm -&gt; gap -6, 121 L, not -76/1,537 L).</t>
+          <t>IN the same branch: IRR_DAILY_TARGET_BY_GH exactly as you wrote; dim.target kept as the cleaning level; Smart Dosing uses the same engine (Pool 1 at 54 cm -&gt; gap -6, 121 L, not -76/1,537 L). | 10:30: gate committed (c2d00ee); the 2 red cases now GREEN on both pages; branch merged to the working branch (4852cb3); PR opened; CI 25 jobs running.</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t>BUILT - NOT YET LIVE</t>
+          <t>IN CI - PR OPEN (merge when green)</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -861,12 +861,12 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>IN the same branch; v21.71 "1 L per 10 cm morning only" rule no longer the default (switch back per pool in Pool &amp; Drum Setup if wanted).</t>
+          <t>IN the same branch; v21.71 "1 L per 10 cm morning only" rule no longer the default (switch back per pool in Pool &amp; Drum Setup if wanted). | 10:30: gate committed (c2d00ee); the 2 red cases now GREEN on both pages; branch merged to the working branch (4852cb3); PR opened; CI 25 jobs running.</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>BUILT - NOT YET LIVE</t>
+          <t>IN CI - PR OPEN (merge when green)</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -911,12 +911,12 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Component finished and judged (3 prototypes, 2 judges); INLINED in the same branch as &lt;script id="hnx-irr-viz-v2222"&gt; in index.html + next.html. Live smoke screenshots taken on the real table (sent to you 07:55). Test "🎛 Gauges" ✓ after the kept-assertion fix.</t>
+          <t>Component finished and judged (3 prototypes, 2 judges); INLINED in the same branch as &lt;script id="hnx-irr-viz-v2222"&gt; in index.html + next.html. Live smoke screenshots taken on the real table (sent to you 07:55). Test "🎛 Gauges" ✓ after the kept-assertion fix. | 10:30: gate committed (c2d00ee); the 2 red cases now GREEN on both pages; branch merged to the working branch (4852cb3); PR opened; CI 25 jobs running.</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t>BUILT - NOT YET LIVE</t>
+          <t>IN CI - PR OPEN (merge when green)</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -961,12 +961,12 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>IN the same branch: engine rewritten (latest reading, Manila day, hold/newer/full gate so a stale computer cannot close a live alarm), old auto calls closed once as "superseded by a newer reading", cards taken down, alarms in the Alerts panel. Tests "🚨 Latest reading only" ✓, "🃏 Stale cards" ✓.</t>
+          <t>IN the same branch: engine rewritten (latest reading, Manila day, hold/newer/full gate so a stale computer cannot close a live alarm), old auto calls closed once as "superseded by a newer reading", cards taken down, alarms in the Alerts panel. Tests "🚨 Latest reading only" ✓, "🃏 Stale cards" ✓. | 10:30: gate committed (c2d00ee); the 2 red cases now GREEN on both pages; branch merged to the working branch (4852cb3); PR opened; CI 25 jobs running.</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>BUILT - NOT YET LIVE</t>
+          <t>IN CI - PR OPEN (merge when green)</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">

</xml_diff>